<commit_message>
Cold outreach Hub step 39: cities go on to their niche's batch
Each niche has one batch, named after it, made when its first city comes.
After the Final check a file is sent on and locked for its sender; in Top
Review a Reviewer sees cities in three lists (Not ready, Ready, Cities
under 10). A city with a Top goes on to the batch an hour later, or at
once with Send to batch now. The same business twice is an error; the
same city twice in a niche is muted until an Owner or Admin unmutes it.
Migration 0027 deletes the batches made before, with their leads.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01B5mxsfamHdKHGSjhV5rcQK
</commit_message>
<xml_diff>
--- a/cold-outreach/hub/e2e/fixtures/top-review.xlsx
+++ b/cold-outreach/hub/e2e/fixtures/top-review.xlsx
@@ -7,7 +7,7 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Tulsa" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Austin" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -481,40 +481,37 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Tulsa Shine 1</t>
+          <t>Austin Shine 1</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>https://share.google/ts1</t>
+          <t>https://share.google/as1</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>100 Main St, Tulsa, OK 74103</t>
+          <t>100 Main St, Austin, TX 78701</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Tulsa</t>
+          <t>Austin</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://tulsashine1.com/</t>
+          <t>https://austinshine1.com/</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>(918) 555-1000</t>
-        </is>
-      </c>
-      <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
-      <c r="I2" t="inlineStr"/>
+          <t>(512) 555-1000</t>
+        </is>
+      </c>
       <c r="J2" t="inlineStr">
         <is>
-          <t>hello@tulsashine1.com</t>
+          <t>hello@austinshine1.com</t>
         </is>
       </c>
       <c r="K2" t="n">
@@ -527,40 +524,37 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Tulsa Shine 2</t>
+          <t>Austin Shine 2</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>https://share.google/ts2</t>
+          <t>https://share.google/as2</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>101 Main St, Tulsa, OK 74103</t>
+          <t>101 Main St, Austin, TX 78701</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Tulsa</t>
+          <t>Austin</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://tulsashine2.com/</t>
+          <t>https://austinshine2.com/</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>(918) 555-1001</t>
-        </is>
-      </c>
-      <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
-      <c r="I3" t="inlineStr"/>
+          <t>(512) 555-1001</t>
+        </is>
+      </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>hello@tulsashine2.com</t>
+          <t>hello@austinshine2.com</t>
         </is>
       </c>
       <c r="K3" t="n">
@@ -573,40 +567,37 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Tulsa Shine 3</t>
+          <t>Austin Shine 3</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>https://share.google/ts3</t>
+          <t>https://share.google/as3</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>102 Main St, Tulsa, OK 74103</t>
+          <t>102 Main St, Austin, TX 78701</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Tulsa</t>
+          <t>Austin</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://tulsashine3.com/</t>
+          <t>https://austinshine3.com/</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>(918) 555-1002</t>
-        </is>
-      </c>
-      <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
-      <c r="I4" t="inlineStr"/>
+          <t>(512) 555-1002</t>
+        </is>
+      </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>hello@tulsashine3.com</t>
+          <t>hello@austinshine3.com</t>
         </is>
       </c>
       <c r="K4" t="n">
@@ -619,40 +610,37 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Tulsa Shine 4</t>
+          <t>Austin Shine 4</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>https://share.google/ts4</t>
+          <t>https://share.google/as4</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>103 Main St, Tulsa, OK 74103</t>
+          <t>103 Main St, Austin, TX 78701</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Tulsa</t>
+          <t>Austin</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://tulsashine4.com/</t>
+          <t>https://austinshine4.com/</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>(918) 555-1003</t>
-        </is>
-      </c>
-      <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
-      <c r="I5" t="inlineStr"/>
+          <t>(512) 555-1003</t>
+        </is>
+      </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>hello@tulsashine4.com</t>
+          <t>hello@austinshine4.com</t>
         </is>
       </c>
       <c r="K5" t="n">
@@ -665,40 +653,37 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Tulsa Shine 5</t>
+          <t>Austin Shine 5</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>https://share.google/ts5</t>
+          <t>https://share.google/as5</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>104 Main St, Tulsa, OK 74103</t>
+          <t>104 Main St, Austin, TX 78701</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Tulsa</t>
+          <t>Austin</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://tulsashine5.com/</t>
+          <t>https://austinshine5.com/</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>(918) 555-1004</t>
-        </is>
-      </c>
-      <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
-      <c r="I6" t="inlineStr"/>
+          <t>(512) 555-1004</t>
+        </is>
+      </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>hello@tulsashine5.com</t>
+          <t>hello@austinshine5.com</t>
         </is>
       </c>
       <c r="K6" t="n">
@@ -711,40 +696,37 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Tulsa Shine 6</t>
+          <t>Austin Shine 6</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>https://share.google/ts6</t>
+          <t>https://share.google/as6</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>105 Main St, Tulsa, OK 74103</t>
+          <t>105 Main St, Austin, TX 78701</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Tulsa</t>
+          <t>Austin</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://tulsashine6.com/</t>
+          <t>https://austinshine6.com/</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>(918) 555-1005</t>
-        </is>
-      </c>
-      <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
-      <c r="I7" t="inlineStr"/>
+          <t>(512) 555-1005</t>
+        </is>
+      </c>
       <c r="J7" t="inlineStr">
         <is>
-          <t>hello@tulsashine6.com</t>
+          <t>hello@austinshine6.com</t>
         </is>
       </c>
       <c r="K7" t="n">
@@ -757,40 +739,37 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Tulsa Shine 7</t>
+          <t>Austin Shine 7</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>https://share.google/ts7</t>
+          <t>https://share.google/as7</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>106 Main St, Tulsa, OK 74103</t>
+          <t>106 Main St, Austin, TX 78701</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Tulsa</t>
+          <t>Austin</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://tulsashine7.com/</t>
+          <t>https://austinshine7.com/</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>(918) 555-1006</t>
-        </is>
-      </c>
-      <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
-      <c r="I8" t="inlineStr"/>
+          <t>(512) 555-1006</t>
+        </is>
+      </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>hello@tulsashine7.com</t>
+          <t>hello@austinshine7.com</t>
         </is>
       </c>
       <c r="K8" t="n">
@@ -803,40 +782,37 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Tulsa Shine 8</t>
+          <t>Austin Shine 8</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>https://share.google/ts8</t>
+          <t>https://share.google/as8</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>107 Main St, Tulsa, OK 74103</t>
+          <t>107 Main St, Austin, TX 78701</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Tulsa</t>
+          <t>Austin</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://tulsashine8.com/</t>
+          <t>https://austinshine8.com/</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>(918) 555-1007</t>
-        </is>
-      </c>
-      <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
-      <c r="I9" t="inlineStr"/>
+          <t>(512) 555-1007</t>
+        </is>
+      </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>hello@tulsashine8.com</t>
+          <t>hello@austinshine8.com</t>
         </is>
       </c>
       <c r="K9" t="n">
@@ -849,40 +825,37 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Tulsa Shine 9</t>
+          <t>Austin Shine 9</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>https://share.google/ts9</t>
+          <t>https://share.google/as9</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>108 Main St, Tulsa, OK 74103</t>
+          <t>108 Main St, Austin, TX 78701</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Tulsa</t>
+          <t>Austin</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://tulsashine9.com/</t>
+          <t>https://austinshine9.com/</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>(918) 555-1008</t>
-        </is>
-      </c>
-      <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
-      <c r="I10" t="inlineStr"/>
+          <t>(512) 555-1008</t>
+        </is>
+      </c>
       <c r="J10" t="inlineStr">
         <is>
-          <t>hello@tulsashine9.com</t>
+          <t>hello@austinshine9.com</t>
         </is>
       </c>
       <c r="K10" t="n">
@@ -895,40 +868,37 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Tulsa Shine 10</t>
+          <t>Austin Shine 10</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>https://share.google/ts10</t>
+          <t>https://share.google/as10</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>109 Main St, Tulsa, OK 74103</t>
+          <t>109 Main St, Austin, TX 78701</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Tulsa</t>
+          <t>Austin</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://tulsashine10.com/</t>
+          <t>https://austinshine10.com/</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>(918) 555-1009</t>
-        </is>
-      </c>
-      <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
-      <c r="I11" t="inlineStr"/>
+          <t>(512) 555-1009</t>
+        </is>
+      </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>hello@tulsashine10.com</t>
+          <t>hello@austinshine10.com</t>
         </is>
       </c>
       <c r="K11" t="n">
@@ -941,40 +911,37 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Tulsa Shine 11</t>
+          <t>Austin Shine 11</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>https://share.google/ts11</t>
+          <t>https://share.google/as11</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>110 Main St, Tulsa, OK 74103</t>
+          <t>110 Main St, Austin, TX 78701</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Tulsa</t>
+          <t>Austin</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://tulsashine11.com/</t>
+          <t>https://austinshine11.com/</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>(918) 555-1010</t>
-        </is>
-      </c>
-      <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
-      <c r="I12" t="inlineStr"/>
+          <t>(512) 555-1010</t>
+        </is>
+      </c>
       <c r="J12" t="inlineStr">
         <is>
-          <t>hello@tulsashine11.com</t>
+          <t>hello@austinshine11.com</t>
         </is>
       </c>
       <c r="K12" t="n">
@@ -987,40 +954,37 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Tulsa Shine 12</t>
+          <t>Austin Shine 12</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>https://share.google/ts12</t>
+          <t>https://share.google/as12</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>111 Main St, Tulsa, OK 74103</t>
+          <t>111 Main St, Austin, TX 78701</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Tulsa</t>
+          <t>Austin</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>https://tulsashine12.com/</t>
+          <t>https://austinshine12.com/</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>(918) 555-1011</t>
-        </is>
-      </c>
-      <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
-      <c r="I13" t="inlineStr"/>
+          <t>(512) 555-1011</t>
+        </is>
+      </c>
       <c r="J13" t="inlineStr">
         <is>
-          <t>hello@tulsashine12.com</t>
+          <t>hello@austinshine12.com</t>
         </is>
       </c>
       <c r="K13" t="n">

</xml_diff>